<commit_message>
updated KLs and ref docs
</commit_message>
<xml_diff>
--- a/reference docs/AML-indicator-KL.xlsx
+++ b/reference docs/AML-indicator-KL.xlsx
@@ -5,26 +5,40 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benjz\repos\IMI-Big-Data-AI-AML-Detection-System\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benjz\repos\IMI-Big-Data-AI-AML-Detection-System\reference docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{226A90AE-CFA2-47DF-AED2-70FC6BB7E1C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{461F5470-3E13-4B81-8F89-8F696AFDC639}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="AML Indicators" sheetId="1" r:id="rId1"/>
-    <sheet name="Legend &amp; Typologies" sheetId="2" r:id="rId2"/>
+    <sheet name="Overview" sheetId="4" r:id="rId1"/>
+    <sheet name="AML Indicators" sheetId="1" r:id="rId2"/>
+    <sheet name="Legend &amp; Typologies" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'AML Indicators'!$A$1:$M$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'AML Indicators'!$A$1:$M$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="663" uniqueCount="342">
   <si>
     <t>Indicator Id</t>
   </si>
@@ -990,13 +1004,130 @@
   </si>
   <si>
     <t>Cross-border capable; no country field in schema</t>
+  </si>
+  <si>
+    <t>Total Indicators</t>
+  </si>
+  <si>
+    <t>High Risk</t>
+  </si>
+  <si>
+    <t>Medium Risk</t>
+  </si>
+  <si>
+    <t>Workbook Contents</t>
+  </si>
+  <si>
+    <t>By_Category</t>
+  </si>
+  <si>
+    <t>Indicators grouped by typology category with subtotals</t>
+  </si>
+  <si>
+    <t>AML Indicator Knowledge Library</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Red Flag Indicators &amp; Typology Database </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <u/>
+        <sz val="13"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>for practical implementation in an AML detection pipeline</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Prototype v1.0  |  Emphasis: Standard AML Typologies  |  Scope: Detectable ML Patterns </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <u/>
+        <sz val="10"/>
+        <color rgb="FFCCCCCC"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>given provided data fields</t>
+    </r>
+  </si>
+  <si>
+    <t>Typologies</t>
+  </si>
+  <si>
+    <t>Low Risk</t>
+  </si>
+  <si>
+    <t>Unused Indicators*</t>
+  </si>
+  <si>
+    <t>AML Indicators</t>
+  </si>
+  <si>
+    <t>Self-contained database subset of 44 AML-implementable indicators</t>
+  </si>
+  <si>
+    <t>Primary use: Model Development</t>
+  </si>
+  <si>
+    <t>Primary use: Model Development, Overview</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">                 *See </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"># Excluded Indicators </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>in '</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="3"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>03 - AML-rule-based-flags.md'</t>
+    </r>
+  </si>
+  <si>
+    <t>- Only indicators feasibly implementable into the specific AML detection pipeline have been extracted from the AML Knowledge Library (V2) with their indicator ID preserved</t>
+  </si>
+  <si>
+    <t>- This database is self-contained: Transaction Types have been limited to the data fields provided for the pipeline, and Co Occuring Indicators is limited to this knowledge library</t>
+  </si>
+  <si>
+    <t>- 5 new general (mostly non-OCG specific) AML typologies have been identified, and the indicators classified under these 5 typologies</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1087,8 +1218,97 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="24"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF444444"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <u/>
+      <sz val="10"/>
+      <color rgb="FFCCCCCC"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="16">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1165,8 +1385,38 @@
         <fgColor rgb="FFFBF0F0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F3864"/>
+        <bgColor rgb="FF333333"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E5090"/>
+        <bgColor rgb="FF1F618D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEEF3FA"/>
+        <bgColor rgb="FFE8F5E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+        <bgColor rgb="FF1F618D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFEEF3FA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1213,11 +1463,90 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E1F2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1F2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E1F2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E1F2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E6"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D7E6"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D7E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D7E6"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D7E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFD0D7E6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D7E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1296,9 +1625,49 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" quotePrefix="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{9A306D85-CBC0-402C-8781-C5481D59FF28}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1597,6 +1966,166 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DBCC9DC-170A-45B9-8810-68D01A96E541}">
+  <sheetPr>
+    <tabColor rgb="FF1F3864"/>
+  </sheetPr>
+  <dimension ref="B2:G16"/>
+  <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="2" style="28" customWidth="1"/>
+    <col min="2" max="2" width="22" style="28" customWidth="1"/>
+    <col min="3" max="3" width="52" style="28" customWidth="1"/>
+    <col min="4" max="6" width="18" style="28" customWidth="1"/>
+    <col min="7" max="7" width="22.453125" style="28" customWidth="1"/>
+    <col min="8" max="16384" width="8.54296875" style="28"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="42" t="s">
+        <v>328</v>
+      </c>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
+    </row>
+    <row r="3" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B3" s="41" t="s">
+        <v>329</v>
+      </c>
+      <c r="C3" s="39"/>
+      <c r="D3" s="39"/>
+      <c r="E3" s="39"/>
+      <c r="F3" s="39"/>
+      <c r="G3" s="39"/>
+    </row>
+    <row r="4" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="40" t="s">
+        <v>330</v>
+      </c>
+      <c r="C4" s="39"/>
+      <c r="D4" s="39"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="39"/>
+    </row>
+    <row r="5" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="6" spans="2:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="38">
+        <v>5</v>
+      </c>
+      <c r="C6" s="38">
+        <v>44</v>
+      </c>
+      <c r="D6" s="38">
+        <v>24</v>
+      </c>
+      <c r="E6" s="38">
+        <v>17</v>
+      </c>
+      <c r="F6" s="38">
+        <v>3</v>
+      </c>
+      <c r="G6" s="38">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="37" t="s">
+        <v>331</v>
+      </c>
+      <c r="C7" s="37" t="s">
+        <v>322</v>
+      </c>
+      <c r="D7" s="37" t="s">
+        <v>323</v>
+      </c>
+      <c r="E7" s="37" t="s">
+        <v>324</v>
+      </c>
+      <c r="F7" s="37" t="s">
+        <v>332</v>
+      </c>
+      <c r="G7" s="37" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" ht="19" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E8" s="43" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" ht="7" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="10" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="36" t="s">
+        <v>325</v>
+      </c>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+    </row>
+    <row r="11" spans="2:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B11" s="32" t="s">
+        <v>334</v>
+      </c>
+      <c r="C11" s="31" t="s">
+        <v>335</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>336</v>
+      </c>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" s="32" t="s">
+        <v>326</v>
+      </c>
+      <c r="C12" s="34" t="s">
+        <v>327</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>337</v>
+      </c>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+    </row>
+    <row r="14" spans="2:7" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="44" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B15" s="44" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B16" s="44" t="s">
+        <v>340</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D12:G12"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B4:G4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3559,7 +4088,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>